<commit_message>
Add consolidated SPb budget and fix template handling
- Build Сводный бюджет СПб from 4 ЖК (Астон.Движение, Астон.Реформа, Милый дом, River Park)
- Use fixed BDR template for consistent row labels across regions
- Treat missing indirect expenses as zero when calculating operating profit and EBITDA
- Support recursive input folders and configurable header labels

Co-authored-by: kpetlin21-bot <kpetlin21-bot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget/output/Сводный бюджет Екатеринбурга.xlsx
+++ b/budget/output/Сводный бюджет Екатеринбурга.xlsx
@@ -6015,7 +6015,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ЖК "Твоя Привелегия"</t>
+          <t>Твоя Привелегия</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -11457,7 +11457,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ЖК "Исеть Парк"</t>
+          <t>Исеть Парк</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -16907,7 +16907,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ЖК "Космонавтов 11"</t>
+          <t>Космонавтов 11</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -22339,7 +22339,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ЖК "Утес"</t>
+          <t>Утес</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Fix #VALUE! in R98/R99 and clean text banners from leaf rows
- R98: wrap all operands in IFERROR(*1,0) to handle '-' string in R94
- R99: wrap in IFERROR to protect against cascade #VALUE!
- Rents: all margin rows wrapped with IFERROR
- clean_leaf_value(): non-numeric text (PlanFact banners) converted to '-'
- Rebuild all 3 budget files: EKB, SPb, SPb-2

Co-authored-by: kpetlin21-bot <kpetlin21-bot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget/output/Сводный бюджет Екатеринбурга.xlsx
+++ b/budget/output/Сводный бюджет Екатеринбурга.xlsx
@@ -2657,35 +2657,35 @@
         </is>
       </c>
       <c r="B44" s="10">
-        <f>IF(B4=0,"-",B43/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B43/B4),"-")</f>
         <v/>
       </c>
       <c r="C44" s="10">
-        <f>IF(C4=0,"-",C43/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C43/C4),"-")</f>
         <v/>
       </c>
       <c r="D44" s="10">
-        <f>IF(D4=0,"-",D43/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D43/D4),"-")</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>IF(E4=0,"-",E43/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E43/E4),"-")</f>
         <v/>
       </c>
       <c r="F44" s="10">
-        <f>IF(F4=0,"-",F43/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F43/F4),"-")</f>
         <v/>
       </c>
       <c r="G44" s="10">
-        <f>IF(G4=0,"-",G43/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G43/G4),"-")</f>
         <v/>
       </c>
       <c r="H44" s="10">
-        <f>IF(H4=0,"-",H43/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H43/H4),"-")</f>
         <v/>
       </c>
       <c r="I44" s="10">
-        <f>IF(I4=0,"-",I43/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I43/I4),"-")</f>
         <v/>
       </c>
       <c r="J44" s="4" t="n"/>
@@ -4507,35 +4507,35 @@
         </is>
       </c>
       <c r="B81" s="10">
-        <f>IF(B4=0,"-",B80/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B80/B4),"-")</f>
         <v/>
       </c>
       <c r="C81" s="10">
-        <f>IF(C4=0,"-",C80/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C80/C4),"-")</f>
         <v/>
       </c>
       <c r="D81" s="10">
-        <f>IF(D4=0,"-",D80/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D80/D4),"-")</f>
         <v/>
       </c>
       <c r="E81" s="10">
-        <f>IF(E4=0,"-",E80/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E80/E4),"-")</f>
         <v/>
       </c>
       <c r="F81" s="10">
-        <f>IF(F4=0,"-",F80/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F80/F4),"-")</f>
         <v/>
       </c>
       <c r="G81" s="10">
-        <f>IF(G4=0,"-",G80/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G80/G4),"-")</f>
         <v/>
       </c>
       <c r="H81" s="10">
-        <f>IF(H4=0,"-",H80/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H80/H4),"-")</f>
         <v/>
       </c>
       <c r="I81" s="10">
-        <f>IF(I4=0,"-",I80/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I80/I4),"-")</f>
         <v/>
       </c>
       <c r="J81" s="4" t="n"/>
@@ -4907,35 +4907,35 @@
         </is>
       </c>
       <c r="B89" s="9">
-        <f>B80+B82-B87</f>
+        <f>B80+IFERROR(B82*1,0)-IFERROR(B87*1,0)</f>
         <v/>
       </c>
       <c r="C89" s="9">
-        <f>C80+C82-C87</f>
+        <f>C80+IFERROR(C82*1,0)-IFERROR(C87*1,0)</f>
         <v/>
       </c>
       <c r="D89" s="9">
-        <f>D80+D82-D87</f>
+        <f>D80+IFERROR(D82*1,0)-IFERROR(D87*1,0)</f>
         <v/>
       </c>
       <c r="E89" s="9">
-        <f>E80+E82-E87</f>
+        <f>E80+IFERROR(E82*1,0)-IFERROR(E87*1,0)</f>
         <v/>
       </c>
       <c r="F89" s="9">
-        <f>F80+F82-F87</f>
+        <f>F80+IFERROR(F82*1,0)-IFERROR(F87*1,0)</f>
         <v/>
       </c>
       <c r="G89" s="9">
-        <f>G80+G82-G87</f>
+        <f>G80+IFERROR(G82*1,0)-IFERROR(G87*1,0)</f>
         <v/>
       </c>
       <c r="H89" s="9">
-        <f>H80+H82-H87</f>
+        <f>H80+IFERROR(H82*1,0)-IFERROR(H87*1,0)</f>
         <v/>
       </c>
       <c r="I89" s="9">
-        <f>I80+I82-I87</f>
+        <f>I80+IFERROR(I82*1,0)-IFERROR(I87*1,0)</f>
         <v/>
       </c>
       <c r="J89" s="4" t="n"/>
@@ -4957,35 +4957,35 @@
         </is>
       </c>
       <c r="B90" s="10">
-        <f>IF(B4=0,"-",B89/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B89/B4),"-")</f>
         <v/>
       </c>
       <c r="C90" s="10">
-        <f>IF(C4=0,"-",C89/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C89/C4),"-")</f>
         <v/>
       </c>
       <c r="D90" s="10">
-        <f>IF(D4=0,"-",D89/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D89/D4),"-")</f>
         <v/>
       </c>
       <c r="E90" s="10">
-        <f>IF(E4=0,"-",E89/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E89/E4),"-")</f>
         <v/>
       </c>
       <c r="F90" s="10">
-        <f>IF(F4=0,"-",F89/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F89/F4),"-")</f>
         <v/>
       </c>
       <c r="G90" s="10">
-        <f>IF(G4=0,"-",G89/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G89/G4),"-")</f>
         <v/>
       </c>
       <c r="H90" s="10">
-        <f>IF(H4=0,"-",H89/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H89/H4),"-")</f>
         <v/>
       </c>
       <c r="I90" s="10">
-        <f>IF(I4=0,"-",I89/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I89/I4),"-")</f>
         <v/>
       </c>
       <c r="J90" s="4" t="n"/>
@@ -5357,35 +5357,35 @@
         </is>
       </c>
       <c r="B98" s="9">
-        <f>B89-B91-B94-B95</f>
+        <f>IFERROR(B89*1,0)-IFERROR(B91*1,0)-IFERROR(B94*1,0)-IFERROR(B95*1,0)</f>
         <v/>
       </c>
       <c r="C98" s="9">
-        <f>C89-C91-C94-C95</f>
+        <f>IFERROR(C89*1,0)-IFERROR(C91*1,0)-IFERROR(C94*1,0)-IFERROR(C95*1,0)</f>
         <v/>
       </c>
       <c r="D98" s="9">
-        <f>D89-D91-D94-D95</f>
+        <f>IFERROR(D89*1,0)-IFERROR(D91*1,0)-IFERROR(D94*1,0)-IFERROR(D95*1,0)</f>
         <v/>
       </c>
       <c r="E98" s="9">
-        <f>E89-E91-E94-E95</f>
+        <f>IFERROR(E89*1,0)-IFERROR(E91*1,0)-IFERROR(E94*1,0)-IFERROR(E95*1,0)</f>
         <v/>
       </c>
       <c r="F98" s="9">
-        <f>F89-F91-F94-F95</f>
+        <f>IFERROR(F89*1,0)-IFERROR(F91*1,0)-IFERROR(F94*1,0)-IFERROR(F95*1,0)</f>
         <v/>
       </c>
       <c r="G98" s="9">
-        <f>G89-G91-G94-G95</f>
+        <f>IFERROR(G89*1,0)-IFERROR(G91*1,0)-IFERROR(G94*1,0)-IFERROR(G95*1,0)</f>
         <v/>
       </c>
       <c r="H98" s="9">
-        <f>H89-H91-H94-H95</f>
+        <f>IFERROR(H89*1,0)-IFERROR(H91*1,0)-IFERROR(H94*1,0)-IFERROR(H95*1,0)</f>
         <v/>
       </c>
       <c r="I98" s="9">
-        <f>I89-I91-I94-I95</f>
+        <f>IFERROR(I89*1,0)-IFERROR(I91*1,0)-IFERROR(I94*1,0)-IFERROR(I95*1,0)</f>
         <v/>
       </c>
       <c r="J98" s="4" t="n"/>
@@ -5407,35 +5407,35 @@
         </is>
       </c>
       <c r="B99" s="10">
-        <f>IF(B4=0,"-",B98/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B98/B4),"-")</f>
         <v/>
       </c>
       <c r="C99" s="10">
-        <f>IF(C4=0,"-",C98/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C98/C4),"-")</f>
         <v/>
       </c>
       <c r="D99" s="10">
-        <f>IF(D4=0,"-",D98/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D98/D4),"-")</f>
         <v/>
       </c>
       <c r="E99" s="10">
-        <f>IF(E4=0,"-",E98/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E98/E4),"-")</f>
         <v/>
       </c>
       <c r="F99" s="10">
-        <f>IF(F4=0,"-",F98/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F98/F4),"-")</f>
         <v/>
       </c>
       <c r="G99" s="10">
-        <f>IF(G4=0,"-",G98/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G98/G4),"-")</f>
         <v/>
       </c>
       <c r="H99" s="10">
-        <f>IF(H4=0,"-",H98/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H98/H4),"-")</f>
         <v/>
       </c>
       <c r="I99" s="10">
-        <f>IF(I4=0,"-",I98/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I98/I4),"-")</f>
         <v/>
       </c>
       <c r="J99" s="4" t="n"/>
@@ -7766,35 +7766,35 @@
         </is>
       </c>
       <c r="B44" s="10">
-        <f>IF(B4=0,"-",B43/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B43/B4),"-")</f>
         <v/>
       </c>
       <c r="C44" s="10">
-        <f>IF(C4=0,"-",C43/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C43/C4),"-")</f>
         <v/>
       </c>
       <c r="D44" s="10">
-        <f>IF(D4=0,"-",D43/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D43/D4),"-")</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>IF(E4=0,"-",E43/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E43/E4),"-")</f>
         <v/>
       </c>
       <c r="F44" s="10">
-        <f>IF(F4=0,"-",F43/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F43/F4),"-")</f>
         <v/>
       </c>
       <c r="G44" s="10">
-        <f>IF(G4=0,"-",G43/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G43/G4),"-")</f>
         <v/>
       </c>
       <c r="H44" s="10">
-        <f>IF(H4=0,"-",H43/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H43/H4),"-")</f>
         <v/>
       </c>
       <c r="I44" s="10">
-        <f>IF(I4=0,"-",I43/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I43/I4),"-")</f>
         <v/>
       </c>
       <c r="J44" s="4" t="n"/>
@@ -9225,18 +9225,42 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Создано с помощью сервиса ПланФакт</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="7" t="n"/>
-      <c r="F70" s="7" t="n"/>
-      <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>Перейти в сервис</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J70" s="4" t="n"/>
@@ -9830,35 +9854,35 @@
         </is>
       </c>
       <c r="B81" s="10">
-        <f>IF(B4=0,"-",B80/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B80/B4),"-")</f>
         <v/>
       </c>
       <c r="C81" s="10">
-        <f>IF(C4=0,"-",C80/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C80/C4),"-")</f>
         <v/>
       </c>
       <c r="D81" s="10">
-        <f>IF(D4=0,"-",D80/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D80/D4),"-")</f>
         <v/>
       </c>
       <c r="E81" s="10">
-        <f>IF(E4=0,"-",E80/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E80/E4),"-")</f>
         <v/>
       </c>
       <c r="F81" s="10">
-        <f>IF(F4=0,"-",F80/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F80/F4),"-")</f>
         <v/>
       </c>
       <c r="G81" s="10">
-        <f>IF(G4=0,"-",G80/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G80/G4),"-")</f>
         <v/>
       </c>
       <c r="H81" s="10">
-        <f>IF(H4=0,"-",H80/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H80/H4),"-")</f>
         <v/>
       </c>
       <c r="I81" s="10">
-        <f>IF(I4=0,"-",I80/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I80/I4),"-")</f>
         <v/>
       </c>
       <c r="J81" s="4" t="n"/>
@@ -10270,35 +10294,35 @@
         </is>
       </c>
       <c r="B89" s="9">
-        <f>B80+B82-B87</f>
+        <f>B80+IFERROR(B82*1,0)-IFERROR(B87*1,0)</f>
         <v/>
       </c>
       <c r="C89" s="9">
-        <f>C80+C82-C87</f>
+        <f>C80+IFERROR(C82*1,0)-IFERROR(C87*1,0)</f>
         <v/>
       </c>
       <c r="D89" s="9">
-        <f>D80+D82-D87</f>
+        <f>D80+IFERROR(D82*1,0)-IFERROR(D87*1,0)</f>
         <v/>
       </c>
       <c r="E89" s="9">
-        <f>E80+E82-E87</f>
+        <f>E80+IFERROR(E82*1,0)-IFERROR(E87*1,0)</f>
         <v/>
       </c>
       <c r="F89" s="9">
-        <f>F80+F82-F87</f>
+        <f>F80+IFERROR(F82*1,0)-IFERROR(F87*1,0)</f>
         <v/>
       </c>
       <c r="G89" s="9">
-        <f>G80+G82-G87</f>
+        <f>G80+IFERROR(G82*1,0)-IFERROR(G87*1,0)</f>
         <v/>
       </c>
       <c r="H89" s="9">
-        <f>H80+H82-H87</f>
+        <f>H80+IFERROR(H82*1,0)-IFERROR(H87*1,0)</f>
         <v/>
       </c>
       <c r="I89" s="9">
-        <f>I80+I82-I87</f>
+        <f>I80+IFERROR(I82*1,0)-IFERROR(I87*1,0)</f>
         <v/>
       </c>
       <c r="J89" s="4" t="n"/>
@@ -10320,35 +10344,35 @@
         </is>
       </c>
       <c r="B90" s="10">
-        <f>IF(B4=0,"-",B89/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B89/B4),"-")</f>
         <v/>
       </c>
       <c r="C90" s="10">
-        <f>IF(C4=0,"-",C89/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C89/C4),"-")</f>
         <v/>
       </c>
       <c r="D90" s="10">
-        <f>IF(D4=0,"-",D89/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D89/D4),"-")</f>
         <v/>
       </c>
       <c r="E90" s="10">
-        <f>IF(E4=0,"-",E89/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E89/E4),"-")</f>
         <v/>
       </c>
       <c r="F90" s="10">
-        <f>IF(F4=0,"-",F89/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F89/F4),"-")</f>
         <v/>
       </c>
       <c r="G90" s="10">
-        <f>IF(G4=0,"-",G89/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G89/G4),"-")</f>
         <v/>
       </c>
       <c r="H90" s="10">
-        <f>IF(H4=0,"-",H89/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H89/H4),"-")</f>
         <v/>
       </c>
       <c r="I90" s="10">
-        <f>IF(I4=0,"-",I89/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I89/I4),"-")</f>
         <v/>
       </c>
       <c r="J90" s="4" t="n"/>
@@ -10740,35 +10764,35 @@
         </is>
       </c>
       <c r="B98" s="9">
-        <f>B89-B91-B94-B95</f>
+        <f>IFERROR(B89*1,0)-IFERROR(B91*1,0)-IFERROR(B94*1,0)-IFERROR(B95*1,0)</f>
         <v/>
       </c>
       <c r="C98" s="9">
-        <f>C89-C91-C94-C95</f>
+        <f>IFERROR(C89*1,0)-IFERROR(C91*1,0)-IFERROR(C94*1,0)-IFERROR(C95*1,0)</f>
         <v/>
       </c>
       <c r="D98" s="9">
-        <f>D89-D91-D94-D95</f>
+        <f>IFERROR(D89*1,0)-IFERROR(D91*1,0)-IFERROR(D94*1,0)-IFERROR(D95*1,0)</f>
         <v/>
       </c>
       <c r="E98" s="9">
-        <f>E89-E91-E94-E95</f>
+        <f>IFERROR(E89*1,0)-IFERROR(E91*1,0)-IFERROR(E94*1,0)-IFERROR(E95*1,0)</f>
         <v/>
       </c>
       <c r="F98" s="9">
-        <f>F89-F91-F94-F95</f>
+        <f>IFERROR(F89*1,0)-IFERROR(F91*1,0)-IFERROR(F94*1,0)-IFERROR(F95*1,0)</f>
         <v/>
       </c>
       <c r="G98" s="9">
-        <f>G89-G91-G94-G95</f>
+        <f>IFERROR(G89*1,0)-IFERROR(G91*1,0)-IFERROR(G94*1,0)-IFERROR(G95*1,0)</f>
         <v/>
       </c>
       <c r="H98" s="9">
-        <f>H89-H91-H94-H95</f>
+        <f>IFERROR(H89*1,0)-IFERROR(H91*1,0)-IFERROR(H94*1,0)-IFERROR(H95*1,0)</f>
         <v/>
       </c>
       <c r="I98" s="9">
-        <f>I89-I91-I94-I95</f>
+        <f>IFERROR(I89*1,0)-IFERROR(I91*1,0)-IFERROR(I94*1,0)-IFERROR(I95*1,0)</f>
         <v/>
       </c>
       <c r="J98" s="4" t="n"/>
@@ -10790,35 +10814,35 @@
         </is>
       </c>
       <c r="B99" s="10">
-        <f>IF(B4=0,"-",B98/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B98/B4),"-")</f>
         <v/>
       </c>
       <c r="C99" s="10">
-        <f>IF(C4=0,"-",C98/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C98/C4),"-")</f>
         <v/>
       </c>
       <c r="D99" s="10">
-        <f>IF(D4=0,"-",D98/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D98/D4),"-")</f>
         <v/>
       </c>
       <c r="E99" s="10">
-        <f>IF(E4=0,"-",E98/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E98/E4),"-")</f>
         <v/>
       </c>
       <c r="F99" s="10">
-        <f>IF(F4=0,"-",F98/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F98/F4),"-")</f>
         <v/>
       </c>
       <c r="G99" s="10">
-        <f>IF(G4=0,"-",G98/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G98/G4),"-")</f>
         <v/>
       </c>
       <c r="H99" s="10">
-        <f>IF(H4=0,"-",H98/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H98/H4),"-")</f>
         <v/>
       </c>
       <c r="I99" s="10">
-        <f>IF(I4=0,"-",I98/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I98/I4),"-")</f>
         <v/>
       </c>
       <c r="J99" s="4" t="n"/>
@@ -13157,35 +13181,35 @@
         </is>
       </c>
       <c r="B44" s="10">
-        <f>IF(B4=0,"-",B43/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B43/B4),"-")</f>
         <v/>
       </c>
       <c r="C44" s="10">
-        <f>IF(C4=0,"-",C43/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C43/C4),"-")</f>
         <v/>
       </c>
       <c r="D44" s="10">
-        <f>IF(D4=0,"-",D43/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D43/D4),"-")</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>IF(E4=0,"-",E43/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E43/E4),"-")</f>
         <v/>
       </c>
       <c r="F44" s="10">
-        <f>IF(F4=0,"-",F43/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F43/F4),"-")</f>
         <v/>
       </c>
       <c r="G44" s="10">
-        <f>IF(G4=0,"-",G43/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G43/G4),"-")</f>
         <v/>
       </c>
       <c r="H44" s="10">
-        <f>IF(H4=0,"-",H43/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H43/H4),"-")</f>
         <v/>
       </c>
       <c r="I44" s="10">
-        <f>IF(I4=0,"-",I43/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I43/I4),"-")</f>
         <v/>
       </c>
       <c r="J44" s="4" t="n"/>
@@ -14616,18 +14640,42 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Создано с помощью сервиса ПланФакт</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="7" t="n"/>
-      <c r="F70" s="7" t="n"/>
-      <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>Перейти в сервис</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J70" s="4" t="n"/>
@@ -15221,35 +15269,35 @@
         </is>
       </c>
       <c r="B81" s="10">
-        <f>IF(B4=0,"-",B80/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B80/B4),"-")</f>
         <v/>
       </c>
       <c r="C81" s="10">
-        <f>IF(C4=0,"-",C80/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C80/C4),"-")</f>
         <v/>
       </c>
       <c r="D81" s="10">
-        <f>IF(D4=0,"-",D80/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D80/D4),"-")</f>
         <v/>
       </c>
       <c r="E81" s="10">
-        <f>IF(E4=0,"-",E80/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E80/E4),"-")</f>
         <v/>
       </c>
       <c r="F81" s="10">
-        <f>IF(F4=0,"-",F80/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F80/F4),"-")</f>
         <v/>
       </c>
       <c r="G81" s="10">
-        <f>IF(G4=0,"-",G80/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G80/G4),"-")</f>
         <v/>
       </c>
       <c r="H81" s="10">
-        <f>IF(H4=0,"-",H80/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H80/H4),"-")</f>
         <v/>
       </c>
       <c r="I81" s="10">
-        <f>IF(I4=0,"-",I80/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I80/I4),"-")</f>
         <v/>
       </c>
       <c r="J81" s="4" t="n"/>
@@ -15661,35 +15709,35 @@
         </is>
       </c>
       <c r="B89" s="9">
-        <f>B80+B82-B87</f>
+        <f>B80+IFERROR(B82*1,0)-IFERROR(B87*1,0)</f>
         <v/>
       </c>
       <c r="C89" s="9">
-        <f>C80+C82-C87</f>
+        <f>C80+IFERROR(C82*1,0)-IFERROR(C87*1,0)</f>
         <v/>
       </c>
       <c r="D89" s="9">
-        <f>D80+D82-D87</f>
+        <f>D80+IFERROR(D82*1,0)-IFERROR(D87*1,0)</f>
         <v/>
       </c>
       <c r="E89" s="9">
-        <f>E80+E82-E87</f>
+        <f>E80+IFERROR(E82*1,0)-IFERROR(E87*1,0)</f>
         <v/>
       </c>
       <c r="F89" s="9">
-        <f>F80+F82-F87</f>
+        <f>F80+IFERROR(F82*1,0)-IFERROR(F87*1,0)</f>
         <v/>
       </c>
       <c r="G89" s="9">
-        <f>G80+G82-G87</f>
+        <f>G80+IFERROR(G82*1,0)-IFERROR(G87*1,0)</f>
         <v/>
       </c>
       <c r="H89" s="9">
-        <f>H80+H82-H87</f>
+        <f>H80+IFERROR(H82*1,0)-IFERROR(H87*1,0)</f>
         <v/>
       </c>
       <c r="I89" s="9">
-        <f>I80+I82-I87</f>
+        <f>I80+IFERROR(I82*1,0)-IFERROR(I87*1,0)</f>
         <v/>
       </c>
       <c r="J89" s="4" t="n"/>
@@ -15711,35 +15759,35 @@
         </is>
       </c>
       <c r="B90" s="10">
-        <f>IF(B4=0,"-",B89/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B89/B4),"-")</f>
         <v/>
       </c>
       <c r="C90" s="10">
-        <f>IF(C4=0,"-",C89/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C89/C4),"-")</f>
         <v/>
       </c>
       <c r="D90" s="10">
-        <f>IF(D4=0,"-",D89/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D89/D4),"-")</f>
         <v/>
       </c>
       <c r="E90" s="10">
-        <f>IF(E4=0,"-",E89/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E89/E4),"-")</f>
         <v/>
       </c>
       <c r="F90" s="10">
-        <f>IF(F4=0,"-",F89/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F89/F4),"-")</f>
         <v/>
       </c>
       <c r="G90" s="10">
-        <f>IF(G4=0,"-",G89/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G89/G4),"-")</f>
         <v/>
       </c>
       <c r="H90" s="10">
-        <f>IF(H4=0,"-",H89/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H89/H4),"-")</f>
         <v/>
       </c>
       <c r="I90" s="10">
-        <f>IF(I4=0,"-",I89/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I89/I4),"-")</f>
         <v/>
       </c>
       <c r="J90" s="4" t="n"/>
@@ -16131,35 +16179,35 @@
         </is>
       </c>
       <c r="B98" s="9">
-        <f>B89-B91-B94-B95</f>
+        <f>IFERROR(B89*1,0)-IFERROR(B91*1,0)-IFERROR(B94*1,0)-IFERROR(B95*1,0)</f>
         <v/>
       </c>
       <c r="C98" s="9">
-        <f>C89-C91-C94-C95</f>
+        <f>IFERROR(C89*1,0)-IFERROR(C91*1,0)-IFERROR(C94*1,0)-IFERROR(C95*1,0)</f>
         <v/>
       </c>
       <c r="D98" s="9">
-        <f>D89-D91-D94-D95</f>
+        <f>IFERROR(D89*1,0)-IFERROR(D91*1,0)-IFERROR(D94*1,0)-IFERROR(D95*1,0)</f>
         <v/>
       </c>
       <c r="E98" s="9">
-        <f>E89-E91-E94-E95</f>
+        <f>IFERROR(E89*1,0)-IFERROR(E91*1,0)-IFERROR(E94*1,0)-IFERROR(E95*1,0)</f>
         <v/>
       </c>
       <c r="F98" s="9">
-        <f>F89-F91-F94-F95</f>
+        <f>IFERROR(F89*1,0)-IFERROR(F91*1,0)-IFERROR(F94*1,0)-IFERROR(F95*1,0)</f>
         <v/>
       </c>
       <c r="G98" s="9">
-        <f>G89-G91-G94-G95</f>
+        <f>IFERROR(G89*1,0)-IFERROR(G91*1,0)-IFERROR(G94*1,0)-IFERROR(G95*1,0)</f>
         <v/>
       </c>
       <c r="H98" s="9">
-        <f>H89-H91-H94-H95</f>
+        <f>IFERROR(H89*1,0)-IFERROR(H91*1,0)-IFERROR(H94*1,0)-IFERROR(H95*1,0)</f>
         <v/>
       </c>
       <c r="I98" s="9">
-        <f>I89-I91-I94-I95</f>
+        <f>IFERROR(I89*1,0)-IFERROR(I91*1,0)-IFERROR(I94*1,0)-IFERROR(I95*1,0)</f>
         <v/>
       </c>
       <c r="J98" s="4" t="n"/>
@@ -16181,35 +16229,35 @@
         </is>
       </c>
       <c r="B99" s="10">
-        <f>IF(B4=0,"-",B98/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B98/B4),"-")</f>
         <v/>
       </c>
       <c r="C99" s="10">
-        <f>IF(C4=0,"-",C98/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C98/C4),"-")</f>
         <v/>
       </c>
       <c r="D99" s="10">
-        <f>IF(D4=0,"-",D98/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D98/D4),"-")</f>
         <v/>
       </c>
       <c r="E99" s="10">
-        <f>IF(E4=0,"-",E98/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E98/E4),"-")</f>
         <v/>
       </c>
       <c r="F99" s="10">
-        <f>IF(F4=0,"-",F98/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F98/F4),"-")</f>
         <v/>
       </c>
       <c r="G99" s="10">
-        <f>IF(G4=0,"-",G98/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G98/G4),"-")</f>
         <v/>
       </c>
       <c r="H99" s="10">
-        <f>IF(H4=0,"-",H98/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H98/H4),"-")</f>
         <v/>
       </c>
       <c r="I99" s="10">
-        <f>IF(I4=0,"-",I98/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I98/I4),"-")</f>
         <v/>
       </c>
       <c r="J99" s="4" t="n"/>
@@ -18560,35 +18608,35 @@
         </is>
       </c>
       <c r="B44" s="10">
-        <f>IF(B4=0,"-",B43/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B43/B4),"-")</f>
         <v/>
       </c>
       <c r="C44" s="10">
-        <f>IF(C4=0,"-",C43/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C43/C4),"-")</f>
         <v/>
       </c>
       <c r="D44" s="10">
-        <f>IF(D4=0,"-",D43/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D43/D4),"-")</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>IF(E4=0,"-",E43/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E43/E4),"-")</f>
         <v/>
       </c>
       <c r="F44" s="10">
-        <f>IF(F4=0,"-",F43/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F43/F4),"-")</f>
         <v/>
       </c>
       <c r="G44" s="10">
-        <f>IF(G4=0,"-",G43/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G43/G4),"-")</f>
         <v/>
       </c>
       <c r="H44" s="10">
-        <f>IF(H4=0,"-",H43/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H43/H4),"-")</f>
         <v/>
       </c>
       <c r="I44" s="10">
-        <f>IF(I4=0,"-",I43/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I43/I4),"-")</f>
         <v/>
       </c>
       <c r="J44" s="4" t="n"/>
@@ -19999,18 +20047,42 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Создано с помощью сервиса ПланФакт</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="7" t="n"/>
-      <c r="F70" s="7" t="n"/>
-      <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>Перейти в сервис</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J70" s="4" t="n"/>
@@ -20604,35 +20676,35 @@
         </is>
       </c>
       <c r="B81" s="10">
-        <f>IF(B4=0,"-",B80/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B80/B4),"-")</f>
         <v/>
       </c>
       <c r="C81" s="10">
-        <f>IF(C4=0,"-",C80/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C80/C4),"-")</f>
         <v/>
       </c>
       <c r="D81" s="10">
-        <f>IF(D4=0,"-",D80/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D80/D4),"-")</f>
         <v/>
       </c>
       <c r="E81" s="10">
-        <f>IF(E4=0,"-",E80/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E80/E4),"-")</f>
         <v/>
       </c>
       <c r="F81" s="10">
-        <f>IF(F4=0,"-",F80/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F80/F4),"-")</f>
         <v/>
       </c>
       <c r="G81" s="10">
-        <f>IF(G4=0,"-",G80/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G80/G4),"-")</f>
         <v/>
       </c>
       <c r="H81" s="10">
-        <f>IF(H4=0,"-",H80/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H80/H4),"-")</f>
         <v/>
       </c>
       <c r="I81" s="10">
-        <f>IF(I4=0,"-",I80/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I80/I4),"-")</f>
         <v/>
       </c>
       <c r="J81" s="4" t="n"/>
@@ -21044,35 +21116,35 @@
         </is>
       </c>
       <c r="B89" s="9">
-        <f>B80+B82-B87</f>
+        <f>B80+IFERROR(B82*1,0)-IFERROR(B87*1,0)</f>
         <v/>
       </c>
       <c r="C89" s="9">
-        <f>C80+C82-C87</f>
+        <f>C80+IFERROR(C82*1,0)-IFERROR(C87*1,0)</f>
         <v/>
       </c>
       <c r="D89" s="9">
-        <f>D80+D82-D87</f>
+        <f>D80+IFERROR(D82*1,0)-IFERROR(D87*1,0)</f>
         <v/>
       </c>
       <c r="E89" s="9">
-        <f>E80+E82-E87</f>
+        <f>E80+IFERROR(E82*1,0)-IFERROR(E87*1,0)</f>
         <v/>
       </c>
       <c r="F89" s="9">
-        <f>F80+F82-F87</f>
+        <f>F80+IFERROR(F82*1,0)-IFERROR(F87*1,0)</f>
         <v/>
       </c>
       <c r="G89" s="9">
-        <f>G80+G82-G87</f>
+        <f>G80+IFERROR(G82*1,0)-IFERROR(G87*1,0)</f>
         <v/>
       </c>
       <c r="H89" s="9">
-        <f>H80+H82-H87</f>
+        <f>H80+IFERROR(H82*1,0)-IFERROR(H87*1,0)</f>
         <v/>
       </c>
       <c r="I89" s="9">
-        <f>I80+I82-I87</f>
+        <f>I80+IFERROR(I82*1,0)-IFERROR(I87*1,0)</f>
         <v/>
       </c>
       <c r="J89" s="4" t="n"/>
@@ -21094,35 +21166,35 @@
         </is>
       </c>
       <c r="B90" s="10">
-        <f>IF(B4=0,"-",B89/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B89/B4),"-")</f>
         <v/>
       </c>
       <c r="C90" s="10">
-        <f>IF(C4=0,"-",C89/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C89/C4),"-")</f>
         <v/>
       </c>
       <c r="D90" s="10">
-        <f>IF(D4=0,"-",D89/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D89/D4),"-")</f>
         <v/>
       </c>
       <c r="E90" s="10">
-        <f>IF(E4=0,"-",E89/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E89/E4),"-")</f>
         <v/>
       </c>
       <c r="F90" s="10">
-        <f>IF(F4=0,"-",F89/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F89/F4),"-")</f>
         <v/>
       </c>
       <c r="G90" s="10">
-        <f>IF(G4=0,"-",G89/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G89/G4),"-")</f>
         <v/>
       </c>
       <c r="H90" s="10">
-        <f>IF(H4=0,"-",H89/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H89/H4),"-")</f>
         <v/>
       </c>
       <c r="I90" s="10">
-        <f>IF(I4=0,"-",I89/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I89/I4),"-")</f>
         <v/>
       </c>
       <c r="J90" s="4" t="n"/>
@@ -21514,35 +21586,35 @@
         </is>
       </c>
       <c r="B98" s="9">
-        <f>B89-B91-B94-B95</f>
+        <f>IFERROR(B89*1,0)-IFERROR(B91*1,0)-IFERROR(B94*1,0)-IFERROR(B95*1,0)</f>
         <v/>
       </c>
       <c r="C98" s="9">
-        <f>C89-C91-C94-C95</f>
+        <f>IFERROR(C89*1,0)-IFERROR(C91*1,0)-IFERROR(C94*1,0)-IFERROR(C95*1,0)</f>
         <v/>
       </c>
       <c r="D98" s="9">
-        <f>D89-D91-D94-D95</f>
+        <f>IFERROR(D89*1,0)-IFERROR(D91*1,0)-IFERROR(D94*1,0)-IFERROR(D95*1,0)</f>
         <v/>
       </c>
       <c r="E98" s="9">
-        <f>E89-E91-E94-E95</f>
+        <f>IFERROR(E89*1,0)-IFERROR(E91*1,0)-IFERROR(E94*1,0)-IFERROR(E95*1,0)</f>
         <v/>
       </c>
       <c r="F98" s="9">
-        <f>F89-F91-F94-F95</f>
+        <f>IFERROR(F89*1,0)-IFERROR(F91*1,0)-IFERROR(F94*1,0)-IFERROR(F95*1,0)</f>
         <v/>
       </c>
       <c r="G98" s="9">
-        <f>G89-G91-G94-G95</f>
+        <f>IFERROR(G89*1,0)-IFERROR(G91*1,0)-IFERROR(G94*1,0)-IFERROR(G95*1,0)</f>
         <v/>
       </c>
       <c r="H98" s="9">
-        <f>H89-H91-H94-H95</f>
+        <f>IFERROR(H89*1,0)-IFERROR(H91*1,0)-IFERROR(H94*1,0)-IFERROR(H95*1,0)</f>
         <v/>
       </c>
       <c r="I98" s="9">
-        <f>I89-I91-I94-I95</f>
+        <f>IFERROR(I89*1,0)-IFERROR(I91*1,0)-IFERROR(I94*1,0)-IFERROR(I95*1,0)</f>
         <v/>
       </c>
       <c r="J98" s="4" t="n"/>
@@ -21564,35 +21636,35 @@
         </is>
       </c>
       <c r="B99" s="10">
-        <f>IF(B4=0,"-",B98/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B98/B4),"-")</f>
         <v/>
       </c>
       <c r="C99" s="10">
-        <f>IF(C4=0,"-",C98/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C98/C4),"-")</f>
         <v/>
       </c>
       <c r="D99" s="10">
-        <f>IF(D4=0,"-",D98/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D98/D4),"-")</f>
         <v/>
       </c>
       <c r="E99" s="10">
-        <f>IF(E4=0,"-",E98/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E98/E4),"-")</f>
         <v/>
       </c>
       <c r="F99" s="10">
-        <f>IF(F4=0,"-",F98/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F98/F4),"-")</f>
         <v/>
       </c>
       <c r="G99" s="10">
-        <f>IF(G4=0,"-",G98/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G98/G4),"-")</f>
         <v/>
       </c>
       <c r="H99" s="10">
-        <f>IF(H4=0,"-",H98/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H98/H4),"-")</f>
         <v/>
       </c>
       <c r="I99" s="10">
-        <f>IF(I4=0,"-",I98/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I98/I4),"-")</f>
         <v/>
       </c>
       <c r="J99" s="4" t="n"/>
@@ -23945,35 +24017,35 @@
         </is>
       </c>
       <c r="B44" s="10">
-        <f>IF(B4=0,"-",B43/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B43/B4),"-")</f>
         <v/>
       </c>
       <c r="C44" s="10">
-        <f>IF(C4=0,"-",C43/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C43/C4),"-")</f>
         <v/>
       </c>
       <c r="D44" s="10">
-        <f>IF(D4=0,"-",D43/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D43/D4),"-")</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>IF(E4=0,"-",E43/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E43/E4),"-")</f>
         <v/>
       </c>
       <c r="F44" s="10">
-        <f>IF(F4=0,"-",F43/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F43/F4),"-")</f>
         <v/>
       </c>
       <c r="G44" s="10">
-        <f>IF(G4=0,"-",G43/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G43/G4),"-")</f>
         <v/>
       </c>
       <c r="H44" s="10">
-        <f>IF(H4=0,"-",H43/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H43/H4),"-")</f>
         <v/>
       </c>
       <c r="I44" s="10">
-        <f>IF(I4=0,"-",I43/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I43/I4),"-")</f>
         <v/>
       </c>
       <c r="J44" s="4" t="n"/>
@@ -25404,18 +25476,42 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Создано с помощью сервиса ПланФакт</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="7" t="n"/>
-      <c r="F70" s="7" t="n"/>
-      <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>Перейти в сервис</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J70" s="4" t="n"/>
@@ -26009,35 +26105,35 @@
         </is>
       </c>
       <c r="B81" s="10">
-        <f>IF(B4=0,"-",B80/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B80/B4),"-")</f>
         <v/>
       </c>
       <c r="C81" s="10">
-        <f>IF(C4=0,"-",C80/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C80/C4),"-")</f>
         <v/>
       </c>
       <c r="D81" s="10">
-        <f>IF(D4=0,"-",D80/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D80/D4),"-")</f>
         <v/>
       </c>
       <c r="E81" s="10">
-        <f>IF(E4=0,"-",E80/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E80/E4),"-")</f>
         <v/>
       </c>
       <c r="F81" s="10">
-        <f>IF(F4=0,"-",F80/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F80/F4),"-")</f>
         <v/>
       </c>
       <c r="G81" s="10">
-        <f>IF(G4=0,"-",G80/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G80/G4),"-")</f>
         <v/>
       </c>
       <c r="H81" s="10">
-        <f>IF(H4=0,"-",H80/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H80/H4),"-")</f>
         <v/>
       </c>
       <c r="I81" s="10">
-        <f>IF(I4=0,"-",I80/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I80/I4),"-")</f>
         <v/>
       </c>
       <c r="J81" s="4" t="n"/>
@@ -26449,35 +26545,35 @@
         </is>
       </c>
       <c r="B89" s="9">
-        <f>B80+B82-B87</f>
+        <f>B80+IFERROR(B82*1,0)-IFERROR(B87*1,0)</f>
         <v/>
       </c>
       <c r="C89" s="9">
-        <f>C80+C82-C87</f>
+        <f>C80+IFERROR(C82*1,0)-IFERROR(C87*1,0)</f>
         <v/>
       </c>
       <c r="D89" s="9">
-        <f>D80+D82-D87</f>
+        <f>D80+IFERROR(D82*1,0)-IFERROR(D87*1,0)</f>
         <v/>
       </c>
       <c r="E89" s="9">
-        <f>E80+E82-E87</f>
+        <f>E80+IFERROR(E82*1,0)-IFERROR(E87*1,0)</f>
         <v/>
       </c>
       <c r="F89" s="9">
-        <f>F80+F82-F87</f>
+        <f>F80+IFERROR(F82*1,0)-IFERROR(F87*1,0)</f>
         <v/>
       </c>
       <c r="G89" s="9">
-        <f>G80+G82-G87</f>
+        <f>G80+IFERROR(G82*1,0)-IFERROR(G87*1,0)</f>
         <v/>
       </c>
       <c r="H89" s="9">
-        <f>H80+H82-H87</f>
+        <f>H80+IFERROR(H82*1,0)-IFERROR(H87*1,0)</f>
         <v/>
       </c>
       <c r="I89" s="9">
-        <f>I80+I82-I87</f>
+        <f>I80+IFERROR(I82*1,0)-IFERROR(I87*1,0)</f>
         <v/>
       </c>
       <c r="J89" s="4" t="n"/>
@@ -26499,35 +26595,35 @@
         </is>
       </c>
       <c r="B90" s="10">
-        <f>IF(B4=0,"-",B89/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B89/B4),"-")</f>
         <v/>
       </c>
       <c r="C90" s="10">
-        <f>IF(C4=0,"-",C89/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C89/C4),"-")</f>
         <v/>
       </c>
       <c r="D90" s="10">
-        <f>IF(D4=0,"-",D89/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D89/D4),"-")</f>
         <v/>
       </c>
       <c r="E90" s="10">
-        <f>IF(E4=0,"-",E89/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E89/E4),"-")</f>
         <v/>
       </c>
       <c r="F90" s="10">
-        <f>IF(F4=0,"-",F89/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F89/F4),"-")</f>
         <v/>
       </c>
       <c r="G90" s="10">
-        <f>IF(G4=0,"-",G89/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G89/G4),"-")</f>
         <v/>
       </c>
       <c r="H90" s="10">
-        <f>IF(H4=0,"-",H89/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H89/H4),"-")</f>
         <v/>
       </c>
       <c r="I90" s="10">
-        <f>IF(I4=0,"-",I89/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I89/I4),"-")</f>
         <v/>
       </c>
       <c r="J90" s="4" t="n"/>
@@ -26919,35 +27015,35 @@
         </is>
       </c>
       <c r="B98" s="9">
-        <f>B89-B91-B94-B95</f>
+        <f>IFERROR(B89*1,0)-IFERROR(B91*1,0)-IFERROR(B94*1,0)-IFERROR(B95*1,0)</f>
         <v/>
       </c>
       <c r="C98" s="9">
-        <f>C89-C91-C94-C95</f>
+        <f>IFERROR(C89*1,0)-IFERROR(C91*1,0)-IFERROR(C94*1,0)-IFERROR(C95*1,0)</f>
         <v/>
       </c>
       <c r="D98" s="9">
-        <f>D89-D91-D94-D95</f>
+        <f>IFERROR(D89*1,0)-IFERROR(D91*1,0)-IFERROR(D94*1,0)-IFERROR(D95*1,0)</f>
         <v/>
       </c>
       <c r="E98" s="9">
-        <f>E89-E91-E94-E95</f>
+        <f>IFERROR(E89*1,0)-IFERROR(E91*1,0)-IFERROR(E94*1,0)-IFERROR(E95*1,0)</f>
         <v/>
       </c>
       <c r="F98" s="9">
-        <f>F89-F91-F94-F95</f>
+        <f>IFERROR(F89*1,0)-IFERROR(F91*1,0)-IFERROR(F94*1,0)-IFERROR(F95*1,0)</f>
         <v/>
       </c>
       <c r="G98" s="9">
-        <f>G89-G91-G94-G95</f>
+        <f>IFERROR(G89*1,0)-IFERROR(G91*1,0)-IFERROR(G94*1,0)-IFERROR(G95*1,0)</f>
         <v/>
       </c>
       <c r="H98" s="9">
-        <f>H89-H91-H94-H95</f>
+        <f>IFERROR(H89*1,0)-IFERROR(H91*1,0)-IFERROR(H94*1,0)-IFERROR(H95*1,0)</f>
         <v/>
       </c>
       <c r="I98" s="9">
-        <f>I89-I91-I94-I95</f>
+        <f>IFERROR(I89*1,0)-IFERROR(I91*1,0)-IFERROR(I94*1,0)-IFERROR(I95*1,0)</f>
         <v/>
       </c>
       <c r="J98" s="4" t="n"/>
@@ -26969,35 +27065,35 @@
         </is>
       </c>
       <c r="B99" s="10">
-        <f>IF(B4=0,"-",B98/B4)</f>
+        <f>IFERROR(IF(B4=0,"-",B98/B4),"-")</f>
         <v/>
       </c>
       <c r="C99" s="10">
-        <f>IF(C4=0,"-",C98/C4)</f>
+        <f>IFERROR(IF(C4=0,"-",C98/C4),"-")</f>
         <v/>
       </c>
       <c r="D99" s="10">
-        <f>IF(D4=0,"-",D98/D4)</f>
+        <f>IFERROR(IF(D4=0,"-",D98/D4),"-")</f>
         <v/>
       </c>
       <c r="E99" s="10">
-        <f>IF(E4=0,"-",E98/E4)</f>
+        <f>IFERROR(IF(E4=0,"-",E98/E4),"-")</f>
         <v/>
       </c>
       <c r="F99" s="10">
-        <f>IF(F4=0,"-",F98/F4)</f>
+        <f>IFERROR(IF(F4=0,"-",F98/F4),"-")</f>
         <v/>
       </c>
       <c r="G99" s="10">
-        <f>IF(G4=0,"-",G98/G4)</f>
+        <f>IFERROR(IF(G4=0,"-",G98/G4),"-")</f>
         <v/>
       </c>
       <c r="H99" s="10">
-        <f>IF(H4=0,"-",H98/H4)</f>
+        <f>IFERROR(IF(H4=0,"-",H98/H4),"-")</f>
         <v/>
       </c>
       <c r="I99" s="10">
-        <f>IF(I4=0,"-",I98/I4)</f>
+        <f>IFERROR(IF(I4=0,"-",I98/I4),"-")</f>
         <v/>
       </c>
       <c r="J99" s="4" t="n"/>

</xml_diff>